<commit_message>
Přidán obrázek pro Pavla, ať může poctivě pracovat. Teoretické vlastnosti modelu dodám později.
</commit_message>
<xml_diff>
--- a/ukol_2/programy/Excel/Program_excel.xlsx
+++ b/ukol_2/programy/Excel/Program_excel.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mapri\Documents\SOP\SOP-2026-A\ukol_2\programy\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vutbr-my.sharepoint.com/personal/257575_vutbr_cz/Documents/Bc-3_2/SOP/SOP-2026-A/ukol_2/programy/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E538C118-5C6F-4B58-A308-907483F58A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="131" documentId="13_ncr:1_{E538C118-5C6F-4B58-A308-907483F58A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A60BF62-946D-4371-8CC7-9B4056711F21}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -196,12 +196,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -516,23 +513,23 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="2"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="1"/>
@@ -541,194 +538,194 @@
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>5</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <v>5</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <v>300</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <v>1</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="6">
         <v>0</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="6">
         <v>50</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <v>0</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="4">
         <v>1</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <v>35</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <v>0.6</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="6">
         <v>1.5</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="6">
         <v>63</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <v>200</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="4">
         <v>350</v>
       </c>
-      <c r="F8" s="5"/>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="3"/>
+      <c r="C9" s="2"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="4">
         <v>30.000000150936849</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="4">
         <v>29.999999849063151</v>
       </c>
-      <c r="F10" s="5"/>
+      <c r="F10" s="4"/>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="3"/>
+      <c r="C11" s="2"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="4">
         <f>D10*D4</f>
         <v>150.00000075468424</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="4">
         <f>E10*E4</f>
         <v>149.99999924531576</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="4">
         <f>SUM(D12:E12)</f>
         <v>300</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="6">
         <f>D10*D5</f>
         <v>30.000000150936849</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="6">
         <f>E10*E5</f>
         <v>0</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="6">
         <f t="shared" ref="F13:F15" si="0">SUM(D13:E13)</f>
         <v>30.000000150936849</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="4">
         <f>D10*D6</f>
         <v>0</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="4">
         <f>E10*E6</f>
         <v>29.999999849063151</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="4">
         <f t="shared" si="0"/>
         <v>29.999999849063151</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="6">
         <f>D10*D7</f>
         <v>18.000000090562107</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="6">
         <f>E10*E7</f>
         <v>44.999999773594723</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="6">
         <f t="shared" si="0"/>
         <v>62.999999864156834</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="4">
         <f>D10*D8</f>
         <v>6000.0000301873697</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="4">
         <f>E10*E8</f>
         <v>10499.999947172102</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="4">
         <f>SUM(D16:E16)</f>
         <v>16499.999977359472</v>
       </c>

</xml_diff>

<commit_message>
Tak je to všechno
</commit_message>
<xml_diff>
--- a/ukol_2/programy/Excel/Program_excel.xlsx
+++ b/ukol_2/programy/Excel/Program_excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vutbr-my.sharepoint.com/personal/257575_vutbr_cz/Documents/Bc-3_2/SOP/SOP-2026-A/ukol_2/programy/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="131" documentId="13_ncr:1_{E538C118-5C6F-4B58-A308-907483F58A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A60BF62-946D-4371-8CC7-9B4056711F21}"/>
+  <xr:revisionPtr revIDLastSave="153" documentId="13_ncr:1_{E538C118-5C6F-4B58-A308-907483F58A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7D1BB9C-2B11-41F4-ADA2-22688FE7A730}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1200" yWindow="1185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -234,6 +234,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>